<commit_message>
Updated CHE_grids model - 2025-09-08 23:17
</commit_message>
<xml_diff>
--- a/VerveStacks_CHE_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_CHE_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHE_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7092DFCA-8917-436B-9E2D-B07E55CE4A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{44B53235-1ABC-423D-8739-C29A0BB40A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2264,7 +2264,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{012C3758-6FD7-41A4-958A-BAFFDB11E51B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88FBB7EC-D7BF-48B3-84A6-6A2EC84CE346}">
   <dimension ref="B2:C184"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>